<commit_message>
Update data and add photo
</commit_message>
<xml_diff>
--- a/조합장 현황.xlsx
+++ b/조합장 현황.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nacfz\Documents\V26\DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD477DA2-1538-4396-A4A0-FA85EDB98697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0FEBD3-7BDB-4E96-BF9C-DF8814ADCDD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10148" uniqueCount="4569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10150" uniqueCount="4571">
   <si>
     <t>전)농협무역 이사(250531), 현)한국배연합회장, 현)한국농협수출협의회장</t>
   </si>
@@ -13733,6 +13733,14 @@
   </si>
   <si>
     <t>전)안강농협 RPC 장장, 전)천북·건천·불국사·양남·현곡농협 전무, 전)경주농협 성동·황성지점장</t>
+    <phoneticPr fontId="16" type="noConversion"/>
+  </si>
+  <si>
+    <t>안수정</t>
+    <phoneticPr fontId="16" type="noConversion"/>
+  </si>
+  <si>
+    <t>전)굴비골농협 이사(9년), 대의원(4년), 전)영광군농민회 법성지회 사무국장, 전)영광군쌀전업농 법성지회 사무국장, 전)법성면 대덕2리 이장</t>
     <phoneticPr fontId="16" type="noConversion"/>
   </si>
 </sst>
@@ -40839,9 +40847,13 @@
       <c r="E605" s="18" t="s">
         <v>2846</v>
       </c>
-      <c r="F605" s="81"/>
+      <c r="F605" s="81" t="s">
+        <v>4569</v>
+      </c>
       <c r="G605" s="18"/>
-      <c r="H605" s="64"/>
+      <c r="H605" s="28" t="s">
+        <v>4570</v>
+      </c>
       <c r="I605" s="41"/>
       <c r="J605" s="20">
         <v>45961</v>

</xml_diff>